<commit_message>
[IMP] sale, purchase: wire base_order mixins and finish order field/method renames
Wire the base_order mixins into sale.order / purchase.order (Phase A: inherit,
dedup identical logic, routing hooks) and propagate the fork's order field and
method renames across all dependent modules:
  order_line -> line_ids
  button_confirm / button_cancel -> action_confirm / action_cancel
  action_quotation_send -> action_send_quotation
  note -> notes
Includes create-time fixes (keep price_unit_auto plain to avoid discount
corruption; drop the product_qty default so precompute runs) and the downstream
test/config adjustments the renames require.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/addons/purchase/static/xls/requests_for_quotation_import_template.xlsx
+++ b/addons/purchase/static/xls/requests_for_quotation_import_template.xlsx
@@ -28,7 +28,7 @@
     <t xml:space="preserve">Vendor*</t>
   </si>
   <si>
-    <t xml:space="preserve">Order Deadline</t>
+    <t xml:space="preserve">Order Date</t>
   </si>
   <si>
     <t xml:space="preserve">Expected Arrival</t>
@@ -91,7 +91,7 @@
     <t xml:space="preserve">P00003</t>
   </si>
   <si>
-    <t xml:space="preserve">Deco Addict</t>
+    <t xml:space="preserve">Acme Corporation</t>
   </si>
   <si>
     <t xml:space="preserve">REF161800</t>

</xml_diff>